<commit_message>
Refresh DQR aggregation publication bundle
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/DQR Multidimensional Aggregation and Evidence-Aware Integration/outputs/aggregation_v2/source_data/DQR_Fig02_source_data.xlsx
+++ b/Project 1 Data Quality Assessment/DQR Multidimensional Aggregation and Evidence-Aware Integration/outputs/aggregation_v2/source_data/DQR_Fig02_source_data.xlsx
@@ -1512,7 +1512,7 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="31" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="23" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
@@ -1667,7 +1667,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>D5_composition</t>
+          <t>within_Full_D5_compositional_contribution</t>
         </is>
       </c>
       <c r="D3" s="2" t="n">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>D5_composition</t>
+          <t>within_Full_D5_compositional_contribution</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
@@ -2003,7 +2003,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>D5_composition</t>
+          <t>within_Full_D5_compositional_contribution</t>
         </is>
       </c>
       <c r="D9" s="2" t="n">

</xml_diff>